<commit_message>
Single cell tester with updated v6 values
</commit_message>
<xml_diff>
--- a/Battery Modeling/Data/HPPC Test/HPPC R_0 MAP.xlsx
+++ b/Battery Modeling/Data/HPPC Test/HPPC R_0 MAP.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\CAR\SP\Formula\Car 26 Vehicle\Vehicle Dynamics\Controls\Battery Modeling\Data\HPPC Test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27B265AF-B7CE-406F-98C5-9D6CFAF3EC5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E3A08B7-96F3-4D53-A691-31910DB0301D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{22DDC590-C9BD-4EB7-8E50-E15A716DEFB6}"/>
+    <workbookView xWindow="31005" yWindow="2235" windowWidth="21600" windowHeight="11295" xr2:uid="{22DDC590-C9BD-4EB7-8E50-E15A716DEFB6}"/>
   </bookViews>
   <sheets>
     <sheet name="ALL" sheetId="10" r:id="rId1"/>
@@ -24,6 +24,7 @@
     <sheet name="3.000154083" sheetId="9" r:id="rId9"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>

</xml_diff>